<commit_message>
Alteração nos Arquivos de Modelo de Artquitetura e Roteiro de Teste
Alteração nos Arquivos de Modelo de Artquitetura e Roteiro de Teste
</commit_message>
<xml_diff>
--- a/4.Teste/INST360 - Roteiro de Teste 1.xlsx
+++ b/4.Teste/INST360 - Roteiro de Teste 1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aluno\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia\OneDrive\Desktop\Coisas do Victor\Instituto-360\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851B84C7-D3D1-4FC1-AE65-777D8E2883B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" tabRatio="913" activeTab="2"/>
+    <workbookView xWindow="2460" yWindow="2460" windowWidth="21600" windowHeight="11385" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
     <definedName name="__xlfn_IFERROR">NA()</definedName>
     <definedName name="combo_SimNao">AUX!$A$2:$A$3</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>Caso de Uso</t>
   </si>
@@ -177,11 +178,14 @@
 email: "breno.silvaa@email.com", 
 senha: 098765;</t>
   </si>
+  <si>
+    <t>.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -832,49 +836,49 @@
     <xf numFmtId="0" fontId="27" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="16" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="15">
-    <cellStyle name="Bom" xfId="1"/>
+    <cellStyle name="Bom" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Cálculo" xfId="2" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Célula de Verificação" xfId="3"/>
+    <cellStyle name="Célula de Verificação" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Entrada" xfId="4" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorreto" xfId="5" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutra" xfId="6"/>
+    <cellStyle name="Neutra" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="7"/>
+    <cellStyle name="Normal 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Nota" xfId="8" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Porcentagem 2" xfId="9"/>
+    <cellStyle name="Porcentagem 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Ruim" xfId="5" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="11" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="12" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título 5" xfId="13"/>
+    <cellStyle name="Título 5" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="Total" xfId="14" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1305,7 +1309,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:L22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1326,18 +1330,18 @@
     <row r="1" spans="2:12" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:12" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="16"/>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="39"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="46"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B3" s="17"/>
@@ -1574,7 +1578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1606,8 +1610,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:W20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.85546875" style="4" bestFit="1" customWidth="1"/>
@@ -1620,58 +1624,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
     </row>
     <row r="2" spans="1:23" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="44">
+      <c r="A2" s="42">
         <v>3</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
     </row>
     <row r="3" spans="1:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="1:23" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="46" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="46"/>
+      <c r="D4" s="44"/>
     </row>
     <row r="5" spans="1:23" ht="282" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="40"/>
+      <c r="D5" s="38"/>
     </row>
     <row r="6" spans="1:23" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="7"/>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="41"/>
+      <c r="D6" s="39"/>
     </row>
     <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1883,6 +1887,11 @@
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>

</xml_diff>

<commit_message>
Adição código fonte e atualização história de usuário
Foi adicionado o código fonte da modelagem do caso de uso "Realizar Cadastro" e também foi atualizado o arquivo de História de Usuário, incluindo imagem do protótipo, atualização também no Roteiro de Teste
</commit_message>
<xml_diff>
--- a/4.Teste/INST360 - Roteiro de Teste 1.xlsx
+++ b/4.Teste/INST360 - Roteiro de Teste 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia\OneDrive\Desktop\Coisas do Victor\Instituto-360\4.Teste\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Desktop\IFSP\Instituto-360\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851B84C7-D3D1-4FC1-AE65-777D8E2883B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B4A5BF-E784-4135-B68F-FA245CEBA830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2460" yWindow="2460" windowWidth="21600" windowHeight="11385" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>Caso de Uso</t>
   </si>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>Realizar cadastro no sistema</t>
-  </si>
-  <si>
-    <t>Para obter sucesso na solicitação de validação de cadastro, a matrícula do usuário não pode já estar cadastrada</t>
   </si>
   <si>
     <t>Mensagem de “Usuário cadastrado com sucesso e aguardando validação”</t>
@@ -1378,13 +1375,13 @@
         <v>3</v>
       </c>
       <c r="F5" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="18"/>
     </row>
@@ -1537,19 +1534,19 @@
       </c>
       <c r="F21" s="3">
         <f>SUM(F5:F19)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
         <f>SUM(G5:G19)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" s="3">
         <f>SUM(H5:H19)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="19">
         <f>SUM(F21:H21)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L21" s="18"/>
     </row>
@@ -1663,7 +1660,7 @@
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" s="38"/>
     </row>
@@ -1709,13 +1706,13 @@
         <v>26</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E9" s="36" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F9" s="32">
         <v>0</v>
@@ -1748,10 +1745,10 @@
         <v>26</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10" s="36" t="s">
         <v>23</v>
@@ -1787,10 +1784,10 @@
         <v>26</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>23</v>
@@ -1890,7 +1887,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizações relacionadas ao modelo de arquitetura
</commit_message>
<xml_diff>
--- a/4.Teste/INST360 - Roteiro de Teste 1.xlsx
+++ b/4.Teste/INST360 - Roteiro de Teste 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Desktop\IFSP\Instituto-360\4.Teste\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia\OneDrive\Desktop\Coisas do Victor\Instituto-360\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B4A5BF-E784-4135-B68F-FA245CEBA830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527D167C-DE81-423D-AAA1-0EBC66A42B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2460" yWindow="2460" windowWidth="21600" windowHeight="11385" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -136,22 +136,6 @@
     <t>Mensagem de “Usuário já cadastrado e em processo de validação"</t>
   </si>
   <si>
-    <t>CREATE DATABASE INST360;
-CREATE TABLE Cadastros (
-    id INT AUTO_INCREMENT PRIMARY KEY,
-    nome VARCHAR(100) NOT NULL,
-    matricula VARCHAR(9) NOT NULL,
-    endereco VARCHAR(255),
-    data_nasc DATE,
-    email VARCHAR(150),
-    data_cad DATETIME DEFAULT CURRENT_TIMESTAMP,
-    senha INT NOT NULL,
-    usuario_valido BOOLEAN DEFAULT FALSE);
-INSERT INTO Cadastros (nome, matricula, endereco, data_nasc, email, senha, usuario_ativo) VALUES 
-(1, 'João Silva', 'SL3050807', 'Rua A, 123 - São Paulo', '1995-06-15', 'joao.silva@email.com', 123456, 1),
-(2, 'Maria Oliveira', 'SL305067X', 'Av. B, 456 - São Paulo', '1998-09-22', 'maria.oliveira@email.com', 654321, 0);</t>
-  </si>
-  <si>
     <t>nome: "João Silva", 
 matricula: "SL3050807", 
 endereco: "Rua A, 123 - São Paulo",
@@ -177,6 +161,22 @@
   </si>
   <si>
     <t>.</t>
+  </si>
+  <si>
+    <t>CREATE DATABASE INST360;
+CREATE TABLE Cadastros (
+    id SERIAL PRIMARY KEY,
+    nome VARCHAR(100) NOT NULL,
+    matricula VARCHAR(9) NOT NULL,
+    endereco VARCHAR(255),
+    data_nasc DATE,
+    email VARCHAR(150),
+    data_cad TIMESTAMP DEFAULT CURRENT_TIMESTAMP,
+    senha VARCHAR(255) NOT NULL,
+    usuario_valido BOOLEAN DEFAULT FALSE);
+INSERT INTO Cadastros (nome, matricula, endereco, data_nasc, email, senha, usuario_ativo) VALUES 
+(1, 'João Silva', 'SL3050807', 'Rua A, 123 - São Paulo', '1995-06-15', 'joao.silva@email.com', 123456, 1),
+(2, 'Maria Oliveira', 'SL305067X', 'Av. B, 456 - São Paulo', '1998-09-22', 'maria.oliveira@email.com', 654321, 0);</t>
   </si>
 </sst>
 </file>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="38" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D5" s="38"/>
     </row>
@@ -1706,7 +1706,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="31" t="s">
         <v>27</v>
@@ -1745,7 +1745,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D10" s="34" t="s">
         <v>28</v>
@@ -1784,7 +1784,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D11" s="34" t="s">
         <v>29</v>
@@ -1887,7 +1887,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update INST360 - Roteiro de Teste 1.xlsx
</commit_message>
<xml_diff>
--- a/4.Teste/INST360 - Roteiro de Teste 1.xlsx
+++ b/4.Teste/INST360 - Roteiro de Teste 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perinav\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia\OneDrive\Desktop\Coisas do Victor\Instituto-360\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EE41A4-A6BE-44CA-AA90-1369079B0BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440F05DF-AA8A-486D-909F-1280EB23E075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2460" yWindow="2460" windowWidth="21600" windowHeight="11385" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -141,8 +141,19 @@
     <t>.</t>
   </si>
   <si>
+    <t>nome: "Maria Oliveira", 
+matricula: "SL3050807", 
+endereco: "Av. B, 456 - São Paulo",
+data_nasc: "1998-09-22", 
+email: "maria.oliveira@email.com", 
+senha: 654321;</t>
+  </si>
+  <si>
+    <t>Mensagem de “Cadastro negado, essa matrícula já está cadastrada!"</t>
+  </si>
+  <si>
     <t>CREATE DATABASE INST360;
-CREATE TABLE Cadastros (
+CREATE TABLE usuarios (
     id SERIAL PRIMARY KEY,
     nome VARCHAR(100) NOT NULL,
     matricula VARCHAR(9) NOT NULL,
@@ -154,17 +165,6 @@
     usuario_valido BOOLEAN DEFAULT FALSE);
 INSERT INTO Cadastros (nome, matricula, endereco, data_nasc, email, senha, usuario_ativo) VALUES 
 (1, 'João Silva', 'SL3050807', 'Rua A, 123 - São Paulo', '1995-06-15', 'joao.silva@email.com', 123456, 1);</t>
-  </si>
-  <si>
-    <t>nome: "Maria Oliveira", 
-matricula: "SL3050807", 
-endereco: "Av. B, 456 - São Paulo",
-data_nasc: "1998-09-22", 
-email: "maria.oliveira@email.com", 
-senha: 654321;</t>
-  </si>
-  <si>
-    <t>Mensagem de “Cadastro negado, essa matrícula já está cadastrada!"</t>
   </si>
 </sst>
 </file>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D5" s="32"/>
     </row>
@@ -1710,10 +1710,10 @@
         <v>26</v>
       </c>
       <c r="C10" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>31</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>32</v>
       </c>
       <c r="E10" s="30" t="s">
         <v>23</v>

</xml_diff>